<commit_message>
Corrected directory of the files.
</commit_message>
<xml_diff>
--- a/xlsx/Power/p1.xlsx
+++ b/xlsx/Power/p1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\36306\Desktop\ERFP_SzilardPalma\Normality test\ReplicationCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10EB5BE9-6D01-4861-9A0C-D1E6F7AF223D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B8C12E-9274-4A40-9A92-830C83D3A486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3420" yWindow="3420" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{E15D2A45-245A-4B67-99D0-7B2747112454}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{E15D2A45-245A-4B67-99D0-7B2747112454}"/>
   </bookViews>
   <sheets>
     <sheet name="Munka1" sheetId="1" r:id="rId1"/>
@@ -404,16 +404,16 @@
         <v>0.85599999999999998</v>
       </c>
       <c r="C1">
-        <v>0.96499999999999997</v>
+        <v>0.85199999999999998</v>
       </c>
       <c r="D1">
-        <v>0.98499999999999999</v>
+        <v>0.96299999999999997</v>
       </c>
       <c r="E1">
-        <v>0.995</v>
+        <v>0.98799999999999999</v>
       </c>
       <c r="F1">
-        <v>1</v>
+        <v>0.999</v>
       </c>
       <c r="G1">
         <v>0.999</v>
@@ -436,13 +436,13 @@
         <v>0.877</v>
       </c>
       <c r="C2">
-        <v>0.97499999999999998</v>
+        <v>0.877</v>
       </c>
       <c r="D2">
-        <v>0.99199999999999999</v>
+        <v>0.97099999999999997</v>
       </c>
       <c r="E2">
-        <v>0.999</v>
+        <v>0.99</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -468,7 +468,7 @@
         <v>0.873</v>
       </c>
       <c r="C3">
-        <v>0.96699999999999997</v>
+        <v>0.97199999999999998</v>
       </c>
       <c r="D3">
         <v>0.99299999999999999</v>
@@ -494,13 +494,13 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>0.64600000000000002</v>
+        <v>0.66700000000000004</v>
       </c>
       <c r="B4">
-        <v>0.873</v>
+        <v>0.876</v>
       </c>
       <c r="C4">
-        <v>0.96399999999999997</v>
+        <v>0.96499999999999997</v>
       </c>
       <c r="D4">
         <v>0.99199999999999999</v>
@@ -532,28 +532,28 @@
         <v>0.20200000000000001</v>
       </c>
       <c r="C5">
-        <v>0.26900000000000002</v>
+        <v>1E-3</v>
       </c>
       <c r="D5">
-        <v>0.38</v>
+        <v>3.5999999999999997E-2</v>
       </c>
       <c r="E5">
-        <v>0.45500000000000002</v>
+        <v>9.7000000000000003E-2</v>
       </c>
       <c r="F5">
-        <v>0.58399999999999996</v>
+        <v>0.221</v>
       </c>
       <c r="G5">
-        <v>0.68</v>
+        <v>0.34100000000000003</v>
       </c>
       <c r="H5">
-        <v>0.72699999999999998</v>
+        <v>0.47299999999999998</v>
       </c>
       <c r="I5">
-        <v>0.8</v>
+        <v>0.61</v>
       </c>
       <c r="J5">
-        <v>0.86399999999999999</v>
+        <v>0.68200000000000005</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -564,13 +564,13 @@
         <v>0.85099999999999998</v>
       </c>
       <c r="C6">
-        <v>0.96699999999999997</v>
+        <v>0.97699999999999998</v>
       </c>
       <c r="D6">
-        <v>0.98199999999999998</v>
+        <v>0.98799999999999999</v>
       </c>
       <c r="E6">
-        <v>0.996</v>
+        <v>0.997</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -596,7 +596,7 @@
         <v>0.84299999999999997</v>
       </c>
       <c r="C7">
-        <v>0.95299999999999996</v>
+        <v>0.95</v>
       </c>
       <c r="D7">
         <v>0.97599999999999998</v>
@@ -628,25 +628,25 @@
         <v>0.754</v>
       </c>
       <c r="C8">
-        <v>0.91200000000000003</v>
+        <v>0.54600000000000004</v>
       </c>
       <c r="D8">
-        <v>0.97</v>
+        <v>0.89600000000000002</v>
       </c>
       <c r="E8">
-        <v>0.98299999999999998</v>
+        <v>0.96799999999999997</v>
       </c>
       <c r="F8">
-        <v>0.998</v>
+        <v>0.99199999999999999</v>
       </c>
       <c r="G8">
-        <v>0.996</v>
+        <v>0.99199999999999999</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>0.999</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0.999</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -660,19 +660,19 @@
         <v>0.63700000000000001</v>
       </c>
       <c r="C9">
-        <v>0.94399999999999995</v>
+        <v>0.98299999999999998</v>
       </c>
       <c r="D9">
-        <v>0.96399999999999997</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>0.97599999999999998</v>
+        <v>0.997</v>
       </c>
       <c r="F9">
-        <v>0.99099999999999999</v>
+        <v>0.998</v>
       </c>
       <c r="G9">
-        <v>0.99299999999999999</v>
+        <v>0.995</v>
       </c>
       <c r="H9">
         <v>0.998</v>
@@ -681,7 +681,7 @@
         <v>0.999</v>
       </c>
       <c r="J9">
-        <v>0.998</v>
+        <v>0.999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>